<commit_message>
Set coal share of forward costs for economic retirement to 1
</commit_message>
<xml_diff>
--- a/InputData/elec/SoFCtMbCtPR/Shr of Fwd Costs that Must be Covered to be Prevent Retirement.xlsx
+++ b/InputData/elec/SoFCtMbCtPR/Shr of Fwd Costs that Must be Covered to be Prevent Retirement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr codeName="현재_통합_문서" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kjh_local\NEXTgroup_local\2025_local\2. EPS\업데이트 파일\eps-southkorea-3.3.1_2025update_v4.0.3\InputData\elec\SoFCtMbCtPR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\SoFCtMbCtPR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9541C3-C216-43DA-9833-DBF43E70A8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2636D6B6-13BD-45A3-A0ED-794BAA95170F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="19240" windowHeight="11270" xr2:uid="{5E78EF81-321F-43F5-B343-4E83A6575A8A}"/>
+    <workbookView xWindow="2700" yWindow="3060" windowWidth="43200" windowHeight="17145" xr2:uid="{5E78EF81-321F-43F5-B343-4E83A6575A8A}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Source:</t>
   </si>
@@ -127,44 +127,17 @@
   </si>
   <si>
     <t>Notes:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In the US, many coal plants are subject to rules requiring them </t>
-  </si>
-  <si>
-    <t>to retrofit to meet enviromental guidelines. This requires</t>
-  </si>
-  <si>
-    <t>a one time investment decision for plant owners. Because we don't</t>
-  </si>
-  <si>
-    <t>track individual plants in the model, we calibrate the share of forward</t>
-  </si>
-  <si>
-    <t xml:space="preserve">costs that must be recovered to represent the additional revenue that is needed to </t>
-  </si>
-  <si>
-    <t>save and pay for these one time investments and apply this across the distribution</t>
-  </si>
-  <si>
-    <t>of plant types. Calibration is done by comparing model results against other sources,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">including Rhodium's ClimateDeck and EIA's Annual Energy Outlook and Electric </t>
-  </si>
-  <si>
-    <t>Power Monthly.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -172,7 +145,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -180,13 +153,13 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -218,7 +191,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -234,7 +207,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -531,15 +504,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31DA106A-E484-4E2B-B3F9-91B326CF3E2A}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -547,52 +520,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="B5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="B6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="B7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="B8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="B9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="B10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="B11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="B12" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="B13" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -607,12 +537,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="34.58203125" customWidth="1"/>
+    <col min="1" max="1" width="34.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
         <v>24</v>
       </c>
@@ -620,15 +550,15 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -636,7 +566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -644,7 +574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -652,7 +582,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -660,7 +590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -668,7 +598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -676,7 +606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -684,7 +614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -692,7 +622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -700,7 +630,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -708,7 +638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -716,7 +646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -724,7 +654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -732,7 +662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -740,7 +670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -748,7 +678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -756,7 +686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -764,7 +694,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:2">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -772,7 +702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:2">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -780,7 +710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:2">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -788,7 +718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -796,7 +726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:2">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -804,7 +734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:2">
       <c r="A25" t="s">
         <v>28</v>
       </c>
@@ -819,6 +749,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -962,15 +901,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -978,13 +908,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00313796-8232-4A46-A1A7-BA54812B352B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75903D36-E21A-476E-BEDE-292264C9887F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75903D36-E21A-476E-BEDE-292264C9887F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00313796-8232-4A46-A1A7-BA54812B352B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E449932-7465-49FF-87F3-D3C46ACC27B0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E449932-7465-49FF-87F3-D3C46ACC27B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>